<commit_message>
Daylight savings time corrections
</commit_message>
<xml_diff>
--- a/ButtonPairCodes.xlsx
+++ b/ButtonPairCodes.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0b58bf48a7331aef/Documents/Arduino/RemotePlugs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="28" documentId="8_{90FE65FA-2C5E-4089-9F54-384E64CC8782}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9A7BB062-9D1D-4F08-B802-659C0D69EBF0}"/>
+  <xr:revisionPtr revIDLastSave="445" documentId="8_{90FE65FA-2C5E-4089-9F54-384E64CC8782}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{57D15369-F708-412F-A876-1F29D4100B11}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="0" windowWidth="29040" windowHeight="17520" xr2:uid="{1CFF0E8F-40E1-4B34-881B-DC122C3AADDE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{1CFF0E8F-40E1-4B34-881B-DC122C3AADDE}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Old" sheetId="1" r:id="rId1"/>
+    <sheet name="New" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>None</t>
   </si>
@@ -49,21 +50,16 @@
   <si>
     <t>Number are added together, unless they're in the same row, in which case it’s both = off + 3</t>
   </si>
+  <si>
+    <t>`</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -79,7 +75,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -96,19 +92,50 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -198,7 +225,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$L$2</c:f>
+              <c:f>Old!$L$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -218,46 +245,44 @@
             <a:sp3d/>
           </c:spPr>
           <c:cat>
-            <c:strRef>
-              <c:f>Sheet1!$A$3:$A$12</c:f>
-              <c:strCache>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v>None</c:v>
+            <c:numRef>
+              <c:f>New!$A$3:$A$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>3</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>5</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>6</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>7</c:v>
-                </c:pt>
-                <c:pt idx="9">
                   <c:v>8</c:v>
                 </c:pt>
-              </c:strCache>
-            </c:strRef>
+              </c:numCache>
+            </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$L$3:$L$12</c:f>
+              <c:f>Old!$L$3:$L$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -278,7 +303,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$M$2</c:f>
+              <c:f>Old!$M$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -299,46 +324,44 @@
             <a:sp3d/>
           </c:spPr>
           <c:cat>
-            <c:strRef>
-              <c:f>Sheet1!$A$3:$A$12</c:f>
-              <c:strCache>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v>None</c:v>
+            <c:numRef>
+              <c:f>New!$A$3:$A$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>3</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>5</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>6</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>7</c:v>
-                </c:pt>
-                <c:pt idx="9">
                   <c:v>8</c:v>
                 </c:pt>
-              </c:strCache>
-            </c:strRef>
+              </c:numCache>
+            </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$M$3:$M$12</c:f>
+              <c:f>Old!$M$3:$M$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -362,7 +385,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$N$2</c:f>
+              <c:f>Old!$N$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -383,46 +406,44 @@
             <a:sp3d/>
           </c:spPr>
           <c:cat>
-            <c:strRef>
-              <c:f>Sheet1!$A$3:$A$12</c:f>
-              <c:strCache>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v>None</c:v>
+            <c:numRef>
+              <c:f>New!$A$3:$A$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>3</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>5</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>6</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>7</c:v>
-                </c:pt>
-                <c:pt idx="9">
                   <c:v>8</c:v>
                 </c:pt>
-              </c:strCache>
-            </c:strRef>
+              </c:numCache>
+            </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$N$3:$N$12</c:f>
+              <c:f>Old!$N$3:$N$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -434,6 +455,9 @@
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>252</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -449,7 +473,7 @@
           <c:order val="3"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$O$2</c:f>
+              <c:f>Old!$O$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -470,46 +494,44 @@
             <a:sp3d/>
           </c:spPr>
           <c:cat>
-            <c:strRef>
-              <c:f>Sheet1!$A$3:$A$12</c:f>
-              <c:strCache>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v>None</c:v>
+            <c:numRef>
+              <c:f>New!$A$3:$A$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>3</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>5</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>6</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>7</c:v>
-                </c:pt>
-                <c:pt idx="9">
                   <c:v>8</c:v>
                 </c:pt>
-              </c:strCache>
-            </c:strRef>
+              </c:numCache>
+            </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$O$3:$O$12</c:f>
+              <c:f>Old!$O$3:$O$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -539,7 +561,7 @@
           <c:order val="4"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$P$2</c:f>
+              <c:f>Old!$P$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -560,46 +582,44 @@
             <a:sp3d/>
           </c:spPr>
           <c:cat>
-            <c:strRef>
-              <c:f>Sheet1!$A$3:$A$12</c:f>
-              <c:strCache>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v>None</c:v>
+            <c:numRef>
+              <c:f>New!$A$3:$A$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>3</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>5</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>6</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>7</c:v>
-                </c:pt>
-                <c:pt idx="9">
                   <c:v>8</c:v>
                 </c:pt>
-              </c:strCache>
-            </c:strRef>
+              </c:numCache>
+            </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$P$3:$P$12</c:f>
+              <c:f>Old!$P$3:$P$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -632,7 +652,7 @@
           <c:order val="5"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$Q$2</c:f>
+              <c:f>Old!$Q$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -653,46 +673,44 @@
             <a:sp3d/>
           </c:spPr>
           <c:cat>
-            <c:strRef>
-              <c:f>Sheet1!$A$3:$A$12</c:f>
-              <c:strCache>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v>None</c:v>
+            <c:numRef>
+              <c:f>New!$A$3:$A$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>3</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>5</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>6</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>7</c:v>
-                </c:pt>
-                <c:pt idx="9">
                   <c:v>8</c:v>
                 </c:pt>
-              </c:strCache>
-            </c:strRef>
+              </c:numCache>
+            </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$Q$3:$Q$12</c:f>
+              <c:f>Old!$Q$3:$Q$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -728,7 +746,7 @@
           <c:order val="6"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$R$2</c:f>
+              <c:f>Old!$R$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -749,46 +767,44 @@
             <a:sp3d/>
           </c:spPr>
           <c:cat>
-            <c:strRef>
-              <c:f>Sheet1!$A$3:$A$12</c:f>
-              <c:strCache>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v>None</c:v>
+            <c:numRef>
+              <c:f>New!$A$3:$A$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>3</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>5</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>6</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>7</c:v>
-                </c:pt>
-                <c:pt idx="9">
                   <c:v>8</c:v>
                 </c:pt>
-              </c:strCache>
-            </c:strRef>
+              </c:numCache>
+            </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$R$3:$R$12</c:f>
+              <c:f>Old!$R$3:$R$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -827,7 +843,7 @@
           <c:order val="7"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$S$2</c:f>
+              <c:f>Old!$S$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -847,46 +863,44 @@
             <a:sp3d/>
           </c:spPr>
           <c:cat>
-            <c:strRef>
-              <c:f>Sheet1!$A$3:$A$12</c:f>
-              <c:strCache>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v>None</c:v>
+            <c:numRef>
+              <c:f>New!$A$3:$A$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>3</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>5</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>6</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>7</c:v>
-                </c:pt>
-                <c:pt idx="9">
                   <c:v>8</c:v>
                 </c:pt>
-              </c:strCache>
-            </c:strRef>
+              </c:numCache>
+            </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$S$3:$S$12</c:f>
+              <c:f>Old!$S$3:$S$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -928,7 +942,7 @@
           <c:order val="8"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$T$2</c:f>
+              <c:f>Old!$T$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -948,46 +962,44 @@
             <a:sp3d/>
           </c:spPr>
           <c:cat>
-            <c:strRef>
-              <c:f>Sheet1!$A$3:$A$12</c:f>
-              <c:strCache>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v>None</c:v>
+            <c:numRef>
+              <c:f>New!$A$3:$A$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>3</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>5</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>6</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>7</c:v>
-                </c:pt>
-                <c:pt idx="9">
                   <c:v>8</c:v>
                 </c:pt>
-              </c:strCache>
-            </c:strRef>
+              </c:numCache>
+            </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$T$3:$T$12</c:f>
+              <c:f>Old!$T$3:$T$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -1032,7 +1044,7 @@
           <c:order val="9"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$U$2</c:f>
+              <c:f>Old!$U$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1052,46 +1064,44 @@
             <a:sp3d/>
           </c:spPr>
           <c:cat>
-            <c:strRef>
-              <c:f>Sheet1!$A$3:$A$12</c:f>
-              <c:strCache>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v>None</c:v>
+            <c:numRef>
+              <c:f>New!$A$3:$A$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>3</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>5</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>6</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>7</c:v>
-                </c:pt>
-                <c:pt idx="9">
                   <c:v>8</c:v>
                 </c:pt>
-              </c:strCache>
-            </c:strRef>
+              </c:numCache>
+            </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$U$3:$U$12</c:f>
+              <c:f>Old!$U$3:$U$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -1634,7 +1644,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$V$2</c:f>
+              <c:f>Old!$V$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1644,46 +1654,44 @@
             </c:strRef>
           </c:tx>
           <c:cat>
-            <c:strRef>
-              <c:f>Sheet1!$A$3:$A$12</c:f>
-              <c:strCache>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v>None</c:v>
+            <c:numRef>
+              <c:f>New!$A$3:$A$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>3</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>5</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>6</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>7</c:v>
-                </c:pt>
-                <c:pt idx="9">
                   <c:v>8</c:v>
                 </c:pt>
-              </c:strCache>
-            </c:strRef>
+              </c:numCache>
+            </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$V$3:$V$12</c:f>
+              <c:f>Old!$V$3:$V$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -1704,7 +1712,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$W$2</c:f>
+              <c:f>Old!$W$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1714,46 +1722,44 @@
             </c:strRef>
           </c:tx>
           <c:cat>
-            <c:strRef>
-              <c:f>Sheet1!$A$3:$A$12</c:f>
-              <c:strCache>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v>None</c:v>
+            <c:numRef>
+              <c:f>New!$A$3:$A$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>3</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>5</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>6</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>7</c:v>
-                </c:pt>
-                <c:pt idx="9">
                   <c:v>8</c:v>
                 </c:pt>
-              </c:strCache>
-            </c:strRef>
+              </c:numCache>
+            </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$W$3:$W$12</c:f>
+              <c:f>Old!$W$3:$W$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -1777,7 +1783,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$X$2</c:f>
+              <c:f>Old!$X$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1787,46 +1793,44 @@
             </c:strRef>
           </c:tx>
           <c:cat>
-            <c:strRef>
-              <c:f>Sheet1!$A$3:$A$12</c:f>
-              <c:strCache>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v>None</c:v>
+            <c:numRef>
+              <c:f>New!$A$3:$A$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>3</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>5</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>6</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>7</c:v>
-                </c:pt>
-                <c:pt idx="9">
                   <c:v>8</c:v>
                 </c:pt>
-              </c:strCache>
-            </c:strRef>
+              </c:numCache>
+            </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$X$3:$X$12</c:f>
+              <c:f>Old!$X$3:$X$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -1853,7 +1857,7 @@
           <c:order val="3"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$Y$2</c:f>
+              <c:f>Old!$Y$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1863,46 +1867,44 @@
             </c:strRef>
           </c:tx>
           <c:cat>
-            <c:strRef>
-              <c:f>Sheet1!$A$3:$A$12</c:f>
-              <c:strCache>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v>None</c:v>
+            <c:numRef>
+              <c:f>New!$A$3:$A$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>3</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>5</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>6</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>7</c:v>
-                </c:pt>
-                <c:pt idx="9">
                   <c:v>8</c:v>
                 </c:pt>
-              </c:strCache>
-            </c:strRef>
+              </c:numCache>
+            </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$Y$3:$Y$12</c:f>
+              <c:f>Old!$Y$3:$Y$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -1932,7 +1934,7 @@
           <c:order val="4"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$Z$2</c:f>
+              <c:f>Old!$Z$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1942,46 +1944,44 @@
             </c:strRef>
           </c:tx>
           <c:cat>
-            <c:strRef>
-              <c:f>Sheet1!$A$3:$A$12</c:f>
-              <c:strCache>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v>None</c:v>
+            <c:numRef>
+              <c:f>New!$A$3:$A$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>3</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>5</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>6</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>7</c:v>
-                </c:pt>
-                <c:pt idx="9">
                   <c:v>8</c:v>
                 </c:pt>
-              </c:strCache>
-            </c:strRef>
+              </c:numCache>
+            </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$Z$3:$Z$12</c:f>
+              <c:f>Old!$Z$3:$Z$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -2014,7 +2014,7 @@
           <c:order val="5"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$AA$2</c:f>
+              <c:f>Old!$AA$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2024,46 +2024,44 @@
             </c:strRef>
           </c:tx>
           <c:cat>
-            <c:strRef>
-              <c:f>Sheet1!$A$3:$A$12</c:f>
-              <c:strCache>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v>None</c:v>
+            <c:numRef>
+              <c:f>New!$A$3:$A$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>3</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>5</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>6</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>7</c:v>
-                </c:pt>
-                <c:pt idx="9">
                   <c:v>8</c:v>
                 </c:pt>
-              </c:strCache>
-            </c:strRef>
+              </c:numCache>
+            </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$AA$3:$AA$12</c:f>
+              <c:f>Old!$AA$3:$AA$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -2099,7 +2097,7 @@
           <c:order val="6"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$AB$2</c:f>
+              <c:f>Old!$AB$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2109,46 +2107,44 @@
             </c:strRef>
           </c:tx>
           <c:cat>
-            <c:strRef>
-              <c:f>Sheet1!$A$3:$A$12</c:f>
-              <c:strCache>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v>None</c:v>
+            <c:numRef>
+              <c:f>New!$A$3:$A$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>3</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>5</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>6</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>7</c:v>
-                </c:pt>
-                <c:pt idx="9">
                   <c:v>8</c:v>
                 </c:pt>
-              </c:strCache>
-            </c:strRef>
+              </c:numCache>
+            </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$AB$3:$AB$12</c:f>
+              <c:f>Old!$AB$3:$AB$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -2187,7 +2183,7 @@
           <c:order val="7"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$AC$2</c:f>
+              <c:f>Old!$AC$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2197,46 +2193,44 @@
             </c:strRef>
           </c:tx>
           <c:cat>
-            <c:strRef>
-              <c:f>Sheet1!$A$3:$A$12</c:f>
-              <c:strCache>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v>None</c:v>
+            <c:numRef>
+              <c:f>New!$A$3:$A$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>3</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>5</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>6</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>7</c:v>
-                </c:pt>
-                <c:pt idx="9">
                   <c:v>8</c:v>
                 </c:pt>
-              </c:strCache>
-            </c:strRef>
+              </c:numCache>
+            </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$AC$3:$AC$12</c:f>
+              <c:f>Old!$AC$3:$AC$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -2278,7 +2272,7 @@
           <c:order val="8"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$AD$2</c:f>
+              <c:f>Old!$AD$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2288,46 +2282,44 @@
             </c:strRef>
           </c:tx>
           <c:cat>
-            <c:strRef>
-              <c:f>Sheet1!$A$3:$A$12</c:f>
-              <c:strCache>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v>None</c:v>
+            <c:numRef>
+              <c:f>New!$A$3:$A$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>3</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>5</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>6</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>7</c:v>
-                </c:pt>
-                <c:pt idx="9">
                   <c:v>8</c:v>
                 </c:pt>
-              </c:strCache>
-            </c:strRef>
+              </c:numCache>
+            </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$AD$3:$AD$12</c:f>
+              <c:f>Old!$AD$3:$AD$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -2372,7 +2364,7 @@
           <c:order val="9"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$AE$2</c:f>
+              <c:f>Old!$AE$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2382,46 +2374,44 @@
             </c:strRef>
           </c:tx>
           <c:cat>
-            <c:strRef>
-              <c:f>Sheet1!$A$3:$A$12</c:f>
-              <c:strCache>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v>None</c:v>
+            <c:numRef>
+              <c:f>New!$A$3:$A$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>3</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>5</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>6</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>7</c:v>
-                </c:pt>
-                <c:pt idx="9">
                   <c:v>8</c:v>
                 </c:pt>
-              </c:strCache>
-            </c:strRef>
+              </c:numCache>
+            </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$AE$3:$AE$12</c:f>
+              <c:f>Old!$AE$3:$AE$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -2831,6 +2821,10 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -3401,7 +3395,7 @@
       <c r="K4">
         <v>1340735</v>
       </c>
-      <c r="M4" s="4">
+      <c r="M4">
         <f t="shared" si="0"/>
         <v>60</v>
       </c>
@@ -3594,10 +3588,10 @@
       <c r="J6">
         <v>1340867</v>
       </c>
-      <c r="K6" s="3">
+      <c r="K6">
         <v>1340879</v>
       </c>
-      <c r="O6" s="4">
+      <c r="O6">
         <f t="shared" si="0"/>
         <v>204</v>
       </c>
@@ -3741,19 +3735,22 @@
       <c r="G8">
         <v>1333007</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8">
         <v>1335043</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8">
         <v>1335103</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8">
         <v>1341187</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8">
         <v>1341199</v>
       </c>
-      <c r="Q8" s="4">
+      <c r="N8" t="s">
+        <v>4</v>
+      </c>
+      <c r="Q8">
         <f t="shared" si="0"/>
         <v>524</v>
       </c>
@@ -3863,13 +3860,13 @@
       <c r="I10">
         <v>1334543</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10">
         <v>1342723</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10">
         <v>1342735</v>
       </c>
-      <c r="S10" s="4">
+      <c r="S10">
         <f t="shared" si="0"/>
         <v>2060</v>
       </c>
@@ -3945,7 +3942,7 @@
       <c r="K12">
         <v>1340687</v>
       </c>
-      <c r="U12" s="4">
+      <c r="U12">
         <f t="shared" si="0"/>
         <v>8204</v>
       </c>
@@ -3955,19 +3952,19 @@
       </c>
     </row>
     <row r="14" spans="1:31" ht="75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A14:D14"/>
   </mergeCells>
   <conditionalFormatting sqref="B3:K3 D5:K5 E6:K6 F7:K7 G8:K8 H9:K9 I10:K10 J11:K11 K12 C4:K4">
-    <cfRule type="colorScale" priority="37">
+    <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -3981,4 +3978,1413 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75CFA154-0203-44D1-86AD-7A84208BE603}">
+  <dimension ref="A1:W24"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="16384" width="9.140625" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="B1" s="3">
+        <f>POWER(2,24)</f>
+        <v>16777216</v>
+      </c>
+    </row>
+    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A2" s="6"/>
+      <c r="B2" s="3">
+        <v>0</v>
+      </c>
+      <c r="C2" s="3">
+        <v>1</v>
+      </c>
+      <c r="D2" s="3">
+        <v>2</v>
+      </c>
+      <c r="E2" s="3">
+        <v>3</v>
+      </c>
+      <c r="F2" s="3">
+        <v>4</v>
+      </c>
+      <c r="G2" s="3">
+        <v>5</v>
+      </c>
+      <c r="H2" s="3">
+        <v>6</v>
+      </c>
+      <c r="I2" s="3">
+        <v>7</v>
+      </c>
+      <c r="J2" s="3">
+        <v>8</v>
+      </c>
+      <c r="K2" s="3">
+        <v>9</v>
+      </c>
+      <c r="M2" s="6"/>
+      <c r="N2" s="3">
+        <v>4</v>
+      </c>
+      <c r="O2" s="3">
+        <v>5</v>
+      </c>
+      <c r="P2" s="3">
+        <v>2</v>
+      </c>
+      <c r="Q2" s="3">
+        <v>3</v>
+      </c>
+      <c r="R2" s="3">
+        <v>8</v>
+      </c>
+      <c r="S2" s="3">
+        <v>9</v>
+      </c>
+      <c r="T2" s="3">
+        <v>0</v>
+      </c>
+      <c r="U2" s="3">
+        <v>1</v>
+      </c>
+      <c r="V2" s="3">
+        <v>6</v>
+      </c>
+      <c r="W2" s="3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A3" s="7">
+        <v>0</v>
+      </c>
+      <c r="B3" s="4">
+        <v>15404668</v>
+      </c>
+      <c r="C3" s="4">
+        <v>15404668</v>
+      </c>
+      <c r="D3" s="4">
+        <v>15404670</v>
+      </c>
+      <c r="E3" s="4">
+        <v>15404670</v>
+      </c>
+      <c r="F3" s="4">
+        <v>15404669</v>
+      </c>
+      <c r="G3" s="4">
+        <v>15404669</v>
+      </c>
+      <c r="H3" s="4">
+        <v>15404669</v>
+      </c>
+      <c r="I3" s="4">
+        <v>15404669</v>
+      </c>
+      <c r="J3" s="4">
+        <v>15404671</v>
+      </c>
+      <c r="K3" s="4">
+        <v>15404671</v>
+      </c>
+      <c r="M3" s="7">
+        <v>4</v>
+      </c>
+      <c r="N3" s="4">
+        <f>F7</f>
+        <v>15404665</v>
+      </c>
+      <c r="O3" s="4">
+        <f>G7</f>
+        <v>15404665</v>
+      </c>
+      <c r="P3" s="4">
+        <f>F5</f>
+        <v>15404667</v>
+      </c>
+      <c r="Q3" s="4">
+        <f>F6</f>
+        <v>15404667</v>
+      </c>
+      <c r="R3" s="4">
+        <f>J7</f>
+        <v>15404667</v>
+      </c>
+      <c r="S3" s="4">
+        <f>K7</f>
+        <v>15404667</v>
+      </c>
+      <c r="T3" s="4">
+        <f>F3</f>
+        <v>15404669</v>
+      </c>
+      <c r="U3" s="4">
+        <f>F4</f>
+        <v>15404669</v>
+      </c>
+      <c r="V3" s="4">
+        <f>H7</f>
+        <v>15404669</v>
+      </c>
+      <c r="W3" s="4">
+        <f>I7</f>
+        <v>15404669</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A4" s="6">
+        <v>1</v>
+      </c>
+      <c r="C4" s="3">
+        <v>15404660</v>
+      </c>
+      <c r="D4" s="3">
+        <v>15404670</v>
+      </c>
+      <c r="E4" s="3">
+        <v>15404662</v>
+      </c>
+      <c r="F4" s="3">
+        <v>15404669</v>
+      </c>
+      <c r="G4" s="3">
+        <v>15404661</v>
+      </c>
+      <c r="H4" s="3">
+        <v>15404669</v>
+      </c>
+      <c r="I4" s="3">
+        <v>15404661</v>
+      </c>
+      <c r="J4" s="3">
+        <v>15404671</v>
+      </c>
+      <c r="K4" s="3">
+        <v>15404663</v>
+      </c>
+      <c r="M4" s="6">
+        <v>5</v>
+      </c>
+      <c r="O4" s="3">
+        <f>G8</f>
+        <v>15404657</v>
+      </c>
+      <c r="P4" s="3">
+        <f>G5</f>
+        <v>15404667</v>
+      </c>
+      <c r="Q4" s="3">
+        <f>G6</f>
+        <v>15404659</v>
+      </c>
+      <c r="R4" s="3">
+        <f>J8</f>
+        <v>15404667</v>
+      </c>
+      <c r="S4" s="5">
+        <f>K8</f>
+        <v>15404659</v>
+      </c>
+      <c r="T4" s="3">
+        <f>G3</f>
+        <v>15404669</v>
+      </c>
+      <c r="U4" s="3">
+        <f>G4</f>
+        <v>15404661</v>
+      </c>
+      <c r="V4" s="3">
+        <f>H8</f>
+        <v>15404669</v>
+      </c>
+      <c r="W4" s="3">
+        <f>I8</f>
+        <v>15404661</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A5" s="6">
+        <v>2</v>
+      </c>
+      <c r="D5" s="3">
+        <v>15404666</v>
+      </c>
+      <c r="E5" s="3">
+        <v>15404666</v>
+      </c>
+      <c r="F5" s="3">
+        <v>15404667</v>
+      </c>
+      <c r="G5" s="3">
+        <v>15404667</v>
+      </c>
+      <c r="H5" s="3">
+        <v>15404671</v>
+      </c>
+      <c r="I5" s="3">
+        <v>15404671</v>
+      </c>
+      <c r="J5" s="3">
+        <v>15404667</v>
+      </c>
+      <c r="K5" s="3">
+        <v>15404667</v>
+      </c>
+      <c r="M5" s="6">
+        <v>2</v>
+      </c>
+      <c r="P5" s="3">
+        <f>D5</f>
+        <v>15404666</v>
+      </c>
+      <c r="Q5" s="3">
+        <f>E5</f>
+        <v>15404666</v>
+      </c>
+      <c r="R5" s="3">
+        <f>J5</f>
+        <v>15404667</v>
+      </c>
+      <c r="S5" s="3">
+        <f>K5</f>
+        <v>15404667</v>
+      </c>
+      <c r="T5" s="3">
+        <f>D3</f>
+        <v>15404670</v>
+      </c>
+      <c r="U5" s="3">
+        <f>D4</f>
+        <v>15404670</v>
+      </c>
+      <c r="V5" s="3">
+        <f>H5</f>
+        <v>15404671</v>
+      </c>
+      <c r="W5" s="3">
+        <f>I5</f>
+        <v>15404671</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A6" s="6">
+        <v>3</v>
+      </c>
+      <c r="E6" s="3">
+        <v>15404658</v>
+      </c>
+      <c r="F6" s="3">
+        <v>15404667</v>
+      </c>
+      <c r="G6" s="3">
+        <v>15404659</v>
+      </c>
+      <c r="H6" s="3">
+        <v>15404671</v>
+      </c>
+      <c r="I6" s="3">
+        <v>15404663</v>
+      </c>
+      <c r="J6" s="3">
+        <v>15404667</v>
+      </c>
+      <c r="K6" s="3">
+        <v>15404659</v>
+      </c>
+      <c r="M6" s="6">
+        <v>3</v>
+      </c>
+      <c r="Q6" s="3">
+        <f>E6</f>
+        <v>15404658</v>
+      </c>
+      <c r="R6" s="3">
+        <f>J6</f>
+        <v>15404667</v>
+      </c>
+      <c r="S6" s="3">
+        <f>K6</f>
+        <v>15404659</v>
+      </c>
+      <c r="T6" s="3">
+        <f>E3</f>
+        <v>15404670</v>
+      </c>
+      <c r="U6" s="3">
+        <f>E4</f>
+        <v>15404662</v>
+      </c>
+      <c r="V6" s="3">
+        <f>H6</f>
+        <v>15404671</v>
+      </c>
+      <c r="W6" s="3">
+        <f>I6</f>
+        <v>15404663</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A7" s="6">
+        <v>4</v>
+      </c>
+      <c r="F7" s="3">
+        <v>15404665</v>
+      </c>
+      <c r="G7" s="3">
+        <v>15404665</v>
+      </c>
+      <c r="H7" s="3">
+        <v>15404669</v>
+      </c>
+      <c r="I7" s="3">
+        <v>15404669</v>
+      </c>
+      <c r="J7" s="3">
+        <v>15404667</v>
+      </c>
+      <c r="K7" s="3">
+        <v>15404667</v>
+      </c>
+      <c r="M7" s="6">
+        <v>8</v>
+      </c>
+      <c r="R7" s="3">
+        <f>J11</f>
+        <v>15404667</v>
+      </c>
+      <c r="S7" s="3">
+        <f>K11</f>
+        <v>15404667</v>
+      </c>
+      <c r="T7" s="3">
+        <f>J3</f>
+        <v>15404671</v>
+      </c>
+      <c r="U7" s="3">
+        <f>J4</f>
+        <v>15404671</v>
+      </c>
+      <c r="V7" s="3">
+        <f>J9</f>
+        <v>15404671</v>
+      </c>
+      <c r="W7" s="3">
+        <f>J10</f>
+        <v>15404671</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A8" s="6">
+        <v>5</v>
+      </c>
+      <c r="G8" s="3">
+        <v>15404657</v>
+      </c>
+      <c r="H8" s="3">
+        <v>15404669</v>
+      </c>
+      <c r="I8" s="3">
+        <v>15404661</v>
+      </c>
+      <c r="J8" s="3">
+        <v>15404667</v>
+      </c>
+      <c r="K8" s="5">
+        <v>15404659</v>
+      </c>
+      <c r="M8" s="6">
+        <v>9</v>
+      </c>
+      <c r="S8" s="3">
+        <f>K12</f>
+        <v>15404659</v>
+      </c>
+      <c r="T8" s="3">
+        <f>K3</f>
+        <v>15404671</v>
+      </c>
+      <c r="U8" s="3">
+        <f>K4</f>
+        <v>15404663</v>
+      </c>
+      <c r="V8" s="3">
+        <f>K9</f>
+        <v>15404671</v>
+      </c>
+      <c r="W8" s="3">
+        <f>K10</f>
+        <v>15404663</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A9" s="6">
+        <v>6</v>
+      </c>
+      <c r="H9" s="3">
+        <v>15404669</v>
+      </c>
+      <c r="I9" s="3">
+        <v>15404669</v>
+      </c>
+      <c r="J9" s="3">
+        <v>15404671</v>
+      </c>
+      <c r="K9" s="3">
+        <v>15404671</v>
+      </c>
+      <c r="M9" s="6">
+        <v>0</v>
+      </c>
+      <c r="T9" s="3">
+        <f>B3</f>
+        <v>15404668</v>
+      </c>
+      <c r="U9" s="3">
+        <f>C3</f>
+        <v>15404668</v>
+      </c>
+      <c r="V9" s="3">
+        <f>H3</f>
+        <v>15404669</v>
+      </c>
+      <c r="W9" s="3">
+        <f>I3</f>
+        <v>15404669</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A10" s="6">
+        <v>7</v>
+      </c>
+      <c r="I10" s="3">
+        <v>15404661</v>
+      </c>
+      <c r="J10" s="3">
+        <v>15404671</v>
+      </c>
+      <c r="K10" s="3">
+        <v>15404663</v>
+      </c>
+      <c r="M10" s="6">
+        <v>1</v>
+      </c>
+      <c r="U10" s="3">
+        <f>C4</f>
+        <v>15404660</v>
+      </c>
+      <c r="V10" s="3">
+        <f>H4</f>
+        <v>15404669</v>
+      </c>
+      <c r="W10" s="3">
+        <f>I4</f>
+        <v>15404661</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A11" s="6">
+        <v>8</v>
+      </c>
+      <c r="J11" s="3">
+        <v>15404667</v>
+      </c>
+      <c r="K11" s="3">
+        <v>15404667</v>
+      </c>
+      <c r="M11" s="6">
+        <v>6</v>
+      </c>
+      <c r="V11" s="3">
+        <f>H9</f>
+        <v>15404669</v>
+      </c>
+      <c r="W11" s="3">
+        <f>I9</f>
+        <v>15404669</v>
+      </c>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A12" s="6">
+        <v>9</v>
+      </c>
+      <c r="K12" s="3">
+        <v>15404659</v>
+      </c>
+      <c r="M12" s="6">
+        <v>7</v>
+      </c>
+      <c r="W12" s="3">
+        <f>I10</f>
+        <v>15404661</v>
+      </c>
+    </row>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="B14" s="3">
+        <v>15404656</v>
+      </c>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="B15" s="3">
+        <f>IF(B3="","",B3-$B$14)</f>
+        <v>12</v>
+      </c>
+      <c r="C15" s="3">
+        <f t="shared" ref="C15:K15" si="0">IF(C3="","",C3-$B$14)</f>
+        <v>12</v>
+      </c>
+      <c r="D15" s="3">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="E15" s="3">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="F15" s="3">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="G15" s="3">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="H15" s="3">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="I15" s="3">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="J15" s="3">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="K15" s="3">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="N15" s="3">
+        <f>IF(N3="","",N3-$B$14)</f>
+        <v>9</v>
+      </c>
+      <c r="O15" s="3">
+        <f t="shared" ref="O15:W15" si="1">IF(O3="","",O3-$B$14)</f>
+        <v>9</v>
+      </c>
+      <c r="P15" s="3">
+        <f t="shared" si="1"/>
+        <v>11</v>
+      </c>
+      <c r="Q15" s="3">
+        <f t="shared" si="1"/>
+        <v>11</v>
+      </c>
+      <c r="R15" s="3">
+        <f t="shared" si="1"/>
+        <v>11</v>
+      </c>
+      <c r="S15" s="3">
+        <f t="shared" si="1"/>
+        <v>11</v>
+      </c>
+      <c r="T15" s="3">
+        <f t="shared" si="1"/>
+        <v>13</v>
+      </c>
+      <c r="U15" s="3">
+        <f t="shared" si="1"/>
+        <v>13</v>
+      </c>
+      <c r="V15" s="3">
+        <f t="shared" si="1"/>
+        <v>13</v>
+      </c>
+      <c r="W15" s="3">
+        <f t="shared" si="1"/>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="B16" s="3" t="str">
+        <f t="shared" ref="B16:K16" si="2">IF(B4="","",B4-$B$14)</f>
+        <v/>
+      </c>
+      <c r="C16" s="3">
+        <f t="shared" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="D16" s="3">
+        <f t="shared" si="2"/>
+        <v>14</v>
+      </c>
+      <c r="E16" s="3">
+        <f t="shared" si="2"/>
+        <v>6</v>
+      </c>
+      <c r="F16" s="3">
+        <f t="shared" si="2"/>
+        <v>13</v>
+      </c>
+      <c r="G16" s="3">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="H16" s="3">
+        <f t="shared" si="2"/>
+        <v>13</v>
+      </c>
+      <c r="I16" s="3">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="J16" s="3">
+        <f t="shared" si="2"/>
+        <v>15</v>
+      </c>
+      <c r="K16" s="3">
+        <f t="shared" si="2"/>
+        <v>7</v>
+      </c>
+      <c r="N16" s="3" t="str">
+        <f t="shared" ref="N16:W16" si="3">IF(N4="","",N4-$B$14)</f>
+        <v/>
+      </c>
+      <c r="O16" s="3">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="P16" s="3">
+        <f t="shared" si="3"/>
+        <v>11</v>
+      </c>
+      <c r="Q16" s="3">
+        <f t="shared" si="3"/>
+        <v>3</v>
+      </c>
+      <c r="R16" s="3">
+        <f t="shared" si="3"/>
+        <v>11</v>
+      </c>
+      <c r="S16" s="3">
+        <f t="shared" si="3"/>
+        <v>3</v>
+      </c>
+      <c r="T16" s="3">
+        <f t="shared" si="3"/>
+        <v>13</v>
+      </c>
+      <c r="U16" s="3">
+        <f t="shared" si="3"/>
+        <v>5</v>
+      </c>
+      <c r="V16" s="3">
+        <f t="shared" si="3"/>
+        <v>13</v>
+      </c>
+      <c r="W16" s="3">
+        <f t="shared" si="3"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B17" s="3" t="str">
+        <f t="shared" ref="B17:K17" si="4">IF(B5="","",B5-$B$14)</f>
+        <v/>
+      </c>
+      <c r="C17" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="D17" s="3">
+        <f t="shared" si="4"/>
+        <v>10</v>
+      </c>
+      <c r="E17" s="3">
+        <f t="shared" si="4"/>
+        <v>10</v>
+      </c>
+      <c r="F17" s="3">
+        <f t="shared" si="4"/>
+        <v>11</v>
+      </c>
+      <c r="G17" s="3">
+        <f t="shared" si="4"/>
+        <v>11</v>
+      </c>
+      <c r="H17" s="3">
+        <f t="shared" si="4"/>
+        <v>15</v>
+      </c>
+      <c r="I17" s="3">
+        <f t="shared" si="4"/>
+        <v>15</v>
+      </c>
+      <c r="J17" s="3">
+        <f t="shared" si="4"/>
+        <v>11</v>
+      </c>
+      <c r="K17" s="3">
+        <f t="shared" si="4"/>
+        <v>11</v>
+      </c>
+      <c r="N17" s="3" t="str">
+        <f t="shared" ref="N17:W17" si="5">IF(N5="","",N5-$B$14)</f>
+        <v/>
+      </c>
+      <c r="O17" s="3" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="P17" s="3">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="Q17" s="3">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="R17" s="3">
+        <f t="shared" si="5"/>
+        <v>11</v>
+      </c>
+      <c r="S17" s="3">
+        <f t="shared" si="5"/>
+        <v>11</v>
+      </c>
+      <c r="T17" s="3">
+        <f t="shared" si="5"/>
+        <v>14</v>
+      </c>
+      <c r="U17" s="3">
+        <f t="shared" si="5"/>
+        <v>14</v>
+      </c>
+      <c r="V17" s="3">
+        <f t="shared" si="5"/>
+        <v>15</v>
+      </c>
+      <c r="W17" s="3">
+        <f t="shared" si="5"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B18" s="3" t="str">
+        <f t="shared" ref="B18:K18" si="6">IF(B6="","",B6-$B$14)</f>
+        <v/>
+      </c>
+      <c r="C18" s="3" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="D18" s="3" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="E18" s="3">
+        <f t="shared" si="6"/>
+        <v>2</v>
+      </c>
+      <c r="F18" s="3">
+        <f t="shared" si="6"/>
+        <v>11</v>
+      </c>
+      <c r="G18" s="3">
+        <f t="shared" si="6"/>
+        <v>3</v>
+      </c>
+      <c r="H18" s="3">
+        <f t="shared" si="6"/>
+        <v>15</v>
+      </c>
+      <c r="I18" s="3">
+        <f t="shared" si="6"/>
+        <v>7</v>
+      </c>
+      <c r="J18" s="3">
+        <f t="shared" si="6"/>
+        <v>11</v>
+      </c>
+      <c r="K18" s="3">
+        <f t="shared" si="6"/>
+        <v>3</v>
+      </c>
+      <c r="N18" s="3" t="str">
+        <f t="shared" ref="N18:W18" si="7">IF(N6="","",N6-$B$14)</f>
+        <v/>
+      </c>
+      <c r="O18" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="P18" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="Q18" s="3">
+        <f t="shared" si="7"/>
+        <v>2</v>
+      </c>
+      <c r="R18" s="3">
+        <f t="shared" si="7"/>
+        <v>11</v>
+      </c>
+      <c r="S18" s="3">
+        <f t="shared" si="7"/>
+        <v>3</v>
+      </c>
+      <c r="T18" s="3">
+        <f t="shared" si="7"/>
+        <v>14</v>
+      </c>
+      <c r="U18" s="3">
+        <f t="shared" si="7"/>
+        <v>6</v>
+      </c>
+      <c r="V18" s="3">
+        <f t="shared" si="7"/>
+        <v>15</v>
+      </c>
+      <c r="W18" s="3">
+        <f t="shared" si="7"/>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B19" s="3" t="str">
+        <f t="shared" ref="B19:K19" si="8">IF(B7="","",B7-$B$14)</f>
+        <v/>
+      </c>
+      <c r="C19" s="3" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="D19" s="3" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="E19" s="3" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="F19" s="3">
+        <f t="shared" si="8"/>
+        <v>9</v>
+      </c>
+      <c r="G19" s="3">
+        <f t="shared" si="8"/>
+        <v>9</v>
+      </c>
+      <c r="H19" s="3">
+        <f t="shared" si="8"/>
+        <v>13</v>
+      </c>
+      <c r="I19" s="3">
+        <f t="shared" si="8"/>
+        <v>13</v>
+      </c>
+      <c r="J19" s="3">
+        <f t="shared" si="8"/>
+        <v>11</v>
+      </c>
+      <c r="K19" s="3">
+        <f t="shared" si="8"/>
+        <v>11</v>
+      </c>
+      <c r="N19" s="3" t="str">
+        <f t="shared" ref="N19:W19" si="9">IF(N7="","",N7-$B$14)</f>
+        <v/>
+      </c>
+      <c r="O19" s="3" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="P19" s="3" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="Q19" s="3" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="R19" s="3">
+        <f t="shared" si="9"/>
+        <v>11</v>
+      </c>
+      <c r="S19" s="3">
+        <f t="shared" si="9"/>
+        <v>11</v>
+      </c>
+      <c r="T19" s="3">
+        <f t="shared" si="9"/>
+        <v>15</v>
+      </c>
+      <c r="U19" s="3">
+        <f t="shared" si="9"/>
+        <v>15</v>
+      </c>
+      <c r="V19" s="3">
+        <f t="shared" si="9"/>
+        <v>15</v>
+      </c>
+      <c r="W19" s="3">
+        <f t="shared" si="9"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B20" s="3" t="str">
+        <f t="shared" ref="B20:K20" si="10">IF(B8="","",B8-$B$14)</f>
+        <v/>
+      </c>
+      <c r="C20" s="3" t="str">
+        <f t="shared" si="10"/>
+        <v/>
+      </c>
+      <c r="D20" s="3" t="str">
+        <f t="shared" si="10"/>
+        <v/>
+      </c>
+      <c r="E20" s="3" t="str">
+        <f t="shared" si="10"/>
+        <v/>
+      </c>
+      <c r="F20" s="3" t="str">
+        <f t="shared" si="10"/>
+        <v/>
+      </c>
+      <c r="G20" s="3">
+        <f t="shared" si="10"/>
+        <v>1</v>
+      </c>
+      <c r="H20" s="3">
+        <f t="shared" si="10"/>
+        <v>13</v>
+      </c>
+      <c r="I20" s="3">
+        <f t="shared" si="10"/>
+        <v>5</v>
+      </c>
+      <c r="J20" s="3">
+        <f t="shared" si="10"/>
+        <v>11</v>
+      </c>
+      <c r="K20" s="3">
+        <f t="shared" si="10"/>
+        <v>3</v>
+      </c>
+      <c r="N20" s="3" t="str">
+        <f t="shared" ref="N20:W20" si="11">IF(N8="","",N8-$B$14)</f>
+        <v/>
+      </c>
+      <c r="O20" s="3" t="str">
+        <f t="shared" si="11"/>
+        <v/>
+      </c>
+      <c r="P20" s="3" t="str">
+        <f t="shared" si="11"/>
+        <v/>
+      </c>
+      <c r="Q20" s="3" t="str">
+        <f t="shared" si="11"/>
+        <v/>
+      </c>
+      <c r="R20" s="3" t="str">
+        <f t="shared" si="11"/>
+        <v/>
+      </c>
+      <c r="S20" s="3">
+        <f t="shared" si="11"/>
+        <v>3</v>
+      </c>
+      <c r="T20" s="3">
+        <f t="shared" si="11"/>
+        <v>15</v>
+      </c>
+      <c r="U20" s="3">
+        <f t="shared" si="11"/>
+        <v>7</v>
+      </c>
+      <c r="V20" s="3">
+        <f t="shared" si="11"/>
+        <v>15</v>
+      </c>
+      <c r="W20" s="3">
+        <f t="shared" si="11"/>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B21" s="3" t="str">
+        <f t="shared" ref="B21:K21" si="12">IF(B9="","",B9-$B$14)</f>
+        <v/>
+      </c>
+      <c r="C21" s="3" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="D21" s="3" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="E21" s="3" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="F21" s="3" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="G21" s="3" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="H21" s="3">
+        <f t="shared" si="12"/>
+        <v>13</v>
+      </c>
+      <c r="I21" s="3">
+        <f t="shared" si="12"/>
+        <v>13</v>
+      </c>
+      <c r="J21" s="3">
+        <f t="shared" si="12"/>
+        <v>15</v>
+      </c>
+      <c r="K21" s="3">
+        <f t="shared" si="12"/>
+        <v>15</v>
+      </c>
+      <c r="N21" s="3" t="str">
+        <f t="shared" ref="N21:W21" si="13">IF(N9="","",N9-$B$14)</f>
+        <v/>
+      </c>
+      <c r="O21" s="3" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="P21" s="3" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="Q21" s="3" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="R21" s="3" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="S21" s="3" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="T21" s="3">
+        <f t="shared" si="13"/>
+        <v>12</v>
+      </c>
+      <c r="U21" s="3">
+        <f t="shared" si="13"/>
+        <v>12</v>
+      </c>
+      <c r="V21" s="3">
+        <f t="shared" si="13"/>
+        <v>13</v>
+      </c>
+      <c r="W21" s="3">
+        <f t="shared" si="13"/>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B22" s="3" t="str">
+        <f t="shared" ref="B22:K22" si="14">IF(B10="","",B10-$B$14)</f>
+        <v/>
+      </c>
+      <c r="C22" s="3" t="str">
+        <f t="shared" si="14"/>
+        <v/>
+      </c>
+      <c r="D22" s="3" t="str">
+        <f t="shared" si="14"/>
+        <v/>
+      </c>
+      <c r="E22" s="3" t="str">
+        <f t="shared" si="14"/>
+        <v/>
+      </c>
+      <c r="F22" s="3" t="str">
+        <f t="shared" si="14"/>
+        <v/>
+      </c>
+      <c r="G22" s="3" t="str">
+        <f t="shared" si="14"/>
+        <v/>
+      </c>
+      <c r="H22" s="3" t="str">
+        <f t="shared" si="14"/>
+        <v/>
+      </c>
+      <c r="I22" s="3">
+        <f t="shared" si="14"/>
+        <v>5</v>
+      </c>
+      <c r="J22" s="3">
+        <f t="shared" si="14"/>
+        <v>15</v>
+      </c>
+      <c r="K22" s="3">
+        <f t="shared" si="14"/>
+        <v>7</v>
+      </c>
+      <c r="N22" s="3" t="str">
+        <f t="shared" ref="N22:W22" si="15">IF(N10="","",N10-$B$14)</f>
+        <v/>
+      </c>
+      <c r="O22" s="3" t="str">
+        <f t="shared" si="15"/>
+        <v/>
+      </c>
+      <c r="P22" s="3" t="str">
+        <f t="shared" si="15"/>
+        <v/>
+      </c>
+      <c r="Q22" s="3" t="str">
+        <f t="shared" si="15"/>
+        <v/>
+      </c>
+      <c r="R22" s="3" t="str">
+        <f t="shared" si="15"/>
+        <v/>
+      </c>
+      <c r="S22" s="3" t="str">
+        <f t="shared" si="15"/>
+        <v/>
+      </c>
+      <c r="T22" s="3" t="str">
+        <f t="shared" si="15"/>
+        <v/>
+      </c>
+      <c r="U22" s="3">
+        <f t="shared" si="15"/>
+        <v>4</v>
+      </c>
+      <c r="V22" s="3">
+        <f t="shared" si="15"/>
+        <v>13</v>
+      </c>
+      <c r="W22" s="3">
+        <f t="shared" si="15"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B23" s="3" t="str">
+        <f t="shared" ref="B23:K23" si="16">IF(B11="","",B11-$B$14)</f>
+        <v/>
+      </c>
+      <c r="C23" s="3" t="str">
+        <f t="shared" si="16"/>
+        <v/>
+      </c>
+      <c r="D23" s="3" t="str">
+        <f t="shared" si="16"/>
+        <v/>
+      </c>
+      <c r="E23" s="3" t="str">
+        <f t="shared" si="16"/>
+        <v/>
+      </c>
+      <c r="F23" s="3" t="str">
+        <f t="shared" si="16"/>
+        <v/>
+      </c>
+      <c r="G23" s="3" t="str">
+        <f t="shared" si="16"/>
+        <v/>
+      </c>
+      <c r="H23" s="3" t="str">
+        <f t="shared" si="16"/>
+        <v/>
+      </c>
+      <c r="I23" s="3" t="str">
+        <f t="shared" si="16"/>
+        <v/>
+      </c>
+      <c r="J23" s="3">
+        <f t="shared" si="16"/>
+        <v>11</v>
+      </c>
+      <c r="K23" s="3">
+        <f t="shared" si="16"/>
+        <v>11</v>
+      </c>
+      <c r="N23" s="3" t="str">
+        <f t="shared" ref="N23:W23" si="17">IF(N11="","",N11-$B$14)</f>
+        <v/>
+      </c>
+      <c r="O23" s="3" t="str">
+        <f t="shared" si="17"/>
+        <v/>
+      </c>
+      <c r="P23" s="3" t="str">
+        <f t="shared" si="17"/>
+        <v/>
+      </c>
+      <c r="Q23" s="3" t="str">
+        <f t="shared" si="17"/>
+        <v/>
+      </c>
+      <c r="R23" s="3" t="str">
+        <f t="shared" si="17"/>
+        <v/>
+      </c>
+      <c r="S23" s="3" t="str">
+        <f t="shared" si="17"/>
+        <v/>
+      </c>
+      <c r="T23" s="3" t="str">
+        <f t="shared" si="17"/>
+        <v/>
+      </c>
+      <c r="U23" s="3" t="str">
+        <f t="shared" si="17"/>
+        <v/>
+      </c>
+      <c r="V23" s="3">
+        <f t="shared" si="17"/>
+        <v>13</v>
+      </c>
+      <c r="W23" s="3">
+        <f t="shared" si="17"/>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="24" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B24" s="3" t="str">
+        <f t="shared" ref="B24:K24" si="18">IF(B12="","",B12-$B$14)</f>
+        <v/>
+      </c>
+      <c r="C24" s="3" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+      <c r="D24" s="3" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+      <c r="E24" s="3" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+      <c r="F24" s="3" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+      <c r="G24" s="3" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+      <c r="H24" s="3" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+      <c r="I24" s="3" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+      <c r="J24" s="3" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+      <c r="K24" s="3">
+        <f t="shared" si="18"/>
+        <v>3</v>
+      </c>
+      <c r="N24" s="3" t="str">
+        <f t="shared" ref="N24:W24" si="19">IF(N12="","",N12-$B$14)</f>
+        <v/>
+      </c>
+      <c r="O24" s="3" t="str">
+        <f t="shared" si="19"/>
+        <v/>
+      </c>
+      <c r="P24" s="3" t="str">
+        <f t="shared" si="19"/>
+        <v/>
+      </c>
+      <c r="Q24" s="3" t="str">
+        <f t="shared" si="19"/>
+        <v/>
+      </c>
+      <c r="R24" s="3" t="str">
+        <f t="shared" si="19"/>
+        <v/>
+      </c>
+      <c r="S24" s="3" t="str">
+        <f t="shared" si="19"/>
+        <v/>
+      </c>
+      <c r="T24" s="3" t="str">
+        <f t="shared" si="19"/>
+        <v/>
+      </c>
+      <c r="U24" s="3" t="str">
+        <f t="shared" si="19"/>
+        <v/>
+      </c>
+      <c r="V24" s="3" t="str">
+        <f t="shared" si="19"/>
+        <v/>
+      </c>
+      <c r="W24" s="3">
+        <f t="shared" si="19"/>
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="B3:K12">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N3:W12">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B15:W24">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>